<commit_message>
Identified 67% of functions of MDOS4 5-29-84 beta SO FAR.
</commit_message>
<xml_diff>
--- a/mdos4/dos4_dev.xlsx
+++ b/mdos4/dos4_dev.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mario\ModernPersonality\research\mdos4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A163DFA9-EE00-4578-8BAE-D7E99D6725C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE4C81C8-8DB9-4FE4-96C8-2925371F7BBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D60C3D67-5246-48E1-B011-E581AAB97D9A}"/>
+    <workbookView xWindow="4320" yWindow="345" windowWidth="21600" windowHeight="11295" xr2:uid="{D60C3D67-5246-48E1-B011-E581AAB97D9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="23">
   <si>
     <t>July 27, 2023</t>
   </si>
@@ -91,14 +91,25 @@
   </si>
   <si>
     <t>Out of 724 found</t>
+  </si>
+  <si>
+    <t>Glorious Military Exercise "Function Identification-2026"</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -126,9 +137,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -649,6 +661,9 @@
       <c r="C15" s="1"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="C16" s="1"/>
     </row>
     <row r="17" spans="3:3" x14ac:dyDescent="0.25">

</xml_diff>